<commit_message>
Add Windows Inno installer and BratanVPN brand icons.
Ship Setup script/build, app/tray icons, and design wordmark drafts; keep status backlog current.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/BratanVPN_status.xlsx
+++ b/docs/BratanVPN_status.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="492" yWindow="564" windowWidth="15036" windowHeight="7884" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Статус MVP" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Сводка" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Статус MVP" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -523,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1526,12 +1526,12 @@
       </c>
       <c r="D40" s="16" t="inlineStr">
         <is>
-          <t>осталось</t>
+          <t>сделано</t>
         </is>
       </c>
       <c r="E40" s="16" t="inlineStr">
         <is>
-          <t>Как Sota Connect: мастер установки, ярлык, Program Files</t>
+          <t>Inno Setup: apps/client/windows/installer/; выход BratanVPN-Setup-1.0.0.exe → Program Files\BratanVPN + ярлыки</t>
         </is>
       </c>
     </row>
@@ -1571,7 +1571,7 @@
       </c>
       <c r="C42" s="16" t="inlineStr">
         <is>
-          <t>Убрать мигание консоли (cmd/PowerShell) при старте</t>
+          <t>Убрать мигание консоли при старте/elevate (чёрное окно cmd/PowerShell на долю секунды)</t>
         </is>
       </c>
       <c r="D42" s="16" t="inlineStr">
@@ -1581,7 +1581,107 @@
       </c>
       <c r="E42" s="16" t="inlineStr">
         <is>
-          <t>Скорее всего краткий Process.run powershell при elevate/pipe; уйти на native</t>
+          <t>Что это: при первом Подключиться Flutter вызывает powershell.exe для UAC (install helper) — Windows мигом показывает чёрную консоль. Не баг VPN, косметика UX. Чинить позже: нативный elevate без PowerShell. Сейчас НЕ делать.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="16" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="16" t="inlineStr">
+        <is>
+          <t>Дизайн / бренд</t>
+        </is>
+      </c>
+      <c r="C43" s="16" t="inlineStr">
+        <is>
+          <t>Разработать официальный логотип BratanVPN</t>
+        </is>
+      </c>
+      <c r="D43" s="16" t="inlineStr">
+        <is>
+          <t>осталось</t>
+        </is>
+      </c>
+      <c r="E43" s="16" t="inlineStr">
+        <is>
+          <t>Подобрать/сделать финальный логотип. Сейчас: временная tray-иконка (B в кольце). Черновики wordmark в docs/bratanvpn_wordmark_drakar*.png — в приложение пока не взяли.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="16" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="16" t="inlineStr">
+        <is>
+          <t>Дизайн / бренд</t>
+        </is>
+      </c>
+      <c r="C44" s="16" t="inlineStr">
+        <is>
+          <t>Подобрать фирменный шрифт (типографика) для BratanVPN</t>
+        </is>
+      </c>
+      <c r="D44" s="16" t="inlineStr">
+        <is>
+          <t>осталось</t>
+        </is>
+      </c>
+      <c r="E44" s="16" t="inlineStr">
+        <is>
+          <t>Подобрать шрифт для названия/UI (ч/б минимализм). Смотрели рунический Drakar/векторный алфавит — это картинка, не .ttf/.otf; нужен легальный шрифт или свой display только для BRATANVPN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="16" t="inlineStr">
+        <is>
+          <t>Клиент / UI</t>
+        </is>
+      </c>
+      <c r="C45" s="16" t="inlineStr">
+        <is>
+          <t>Временная tray-иконка (черно-белая B)</t>
+        </is>
+      </c>
+      <c r="D45" s="16" t="inlineStr">
+        <is>
+          <t>сделано</t>
+        </is>
+      </c>
+      <c r="E45" s="16" t="inlineStr">
+        <is>
+          <t>apps/client/assets/tray_icon.ico; placeholder до финального логотипа</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="16" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="16" t="inlineStr">
+        <is>
+          <t>Клиент / раздача</t>
+        </is>
+      </c>
+      <c r="C46" s="16" t="inlineStr">
+        <is>
+          <t>Полировка мастера Inno (тексты + баннер + иконка)</t>
+        </is>
+      </c>
+      <c r="D46" s="16" t="inlineStr">
+        <is>
+          <t>сделано</t>
+        </is>
+      </c>
+      <c r="E46" s="16" t="inlineStr">
+        <is>
+          <t>Свои wizard BMP, короткие русские тексты, SetupIcon из tray_icon</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1722,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3">
@@ -1642,7 +1742,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -1672,7 +1772,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8">
@@ -1683,7 +1783,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
     </row>
@@ -1695,7 +1795,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Frameless UI: чёлка убрана, крестик справа / настройки слева</t>
+          <t>Логотип + шрифт уже в Excel (#42, #43); wordmark в UI пробовали и откатили</t>
         </is>
       </c>
     </row>
@@ -1707,7 +1807,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Далее: Inno Setup .exe → Program Files; SmartScreen/подпись; убрать flash консоли</t>
+          <t>Далее: логотип; шрифт; SmartScreen/подпись; push GitHub; Android</t>
         </is>
       </c>
     </row>

</xml_diff>